<commit_message>
fix: replace pd.isna with np.isfinite in equity profile to handle inf values
Prevents ValueError: Out of range float values are not JSON compliant
when MFI/Bias indicators produce inf due to zero denominators.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/AAII_History.xlsx
+++ b/data/AAII_History.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1384"/>
+  <dimension ref="A1:E1389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26732,6 +26732,101 @@
         <v>5.299999999999997</v>
       </c>
     </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B1385" t="n">
+        <v>0.393</v>
+      </c>
+      <c r="C1385" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="D1385" t="n">
+        <v>0.366</v>
+      </c>
+      <c r="E1385" t="n">
+        <v>2.699999999999996</v>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B1386" t="n">
+        <v>0.317</v>
+      </c>
+      <c r="C1386" t="n">
+        <v>0.247</v>
+      </c>
+      <c r="D1386" t="n">
+        <v>0.436</v>
+      </c>
+      <c r="E1386" t="n">
+        <v>-11.9</v>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B1387" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="C1387" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="D1387" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="E1387" t="n">
+        <v>-6.299999999999997</v>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B1388" t="n">
+        <v>0.363</v>
+      </c>
+      <c r="C1388" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="D1388" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="E1388" t="n">
+        <v>-0.7000000000000028</v>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B1389" t="n">
+        <v>0.304</v>
+      </c>
+      <c r="C1389" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D1389" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="E1389" t="n">
+        <v>-17.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>